<commit_message>
Fix expenses import: replace df.columns with row.keys() in import_project_financial
</commit_message>
<xml_diff>
--- a/templates/financial_template.xlsx
+++ b/templates/financial_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\stuff\web\CRM CAE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3967BA3-545E-4346-9880-B6947664B0A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14A16A8-11C0-4005-AD65-2124D81BAF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,14 @@
     <sheet name="Devis actuel" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'suivi chantier'!$A$1:$E$7</definedName>
-    <definedName name="Z_EB2A1D5B_713C_4666_81AF_FB92ADEAC89B_.wvu.FilterData" localSheetId="0" hidden="1">'suivi chantier'!$A$1:$E$7</definedName>
-    <definedName name="Z_F62B73B1_1F1A_486D_90D1_651B959F68DF_.wvu.FilterData" localSheetId="0" hidden="1">'suivi chantier'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'suivi chantier'!$A$1:$E$65</definedName>
+    <definedName name="Z_EB2A1D5B_713C_4666_81AF_FB92ADEAC89B_.wvu.FilterData" localSheetId="0" hidden="1">'suivi chantier'!$A$1:$E$65</definedName>
+    <definedName name="Z_F62B73B1_1F1A_486D_90D1_651B959F68DF_.wvu.FilterData" localSheetId="0" hidden="1">'suivi chantier'!$A$1:$E$65</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Group by Date" guid="{F62B73B1-1F1A-486D-90D1-651B959F68DF}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Group by Catégorie" guid="{EB2A1D5B-713C-4666-81AF-FB92ADEAC89B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Group by Date" guid="{F62B73B1-1F1A-486D-90D1-651B959F68DF}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -48,6 +48,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">à rectifier
@@ -62,6 +63,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">3 déja achété
@@ -74,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="116">
   <si>
     <t>Date</t>
   </si>
@@ -110,9 +112,6 @@
   </si>
   <si>
     <t>Matériau</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 Sac </t>
   </si>
   <si>
     <t>100 Pieces</t>
@@ -286,22 +285,163 @@
     <t>Total TTC</t>
   </si>
   <si>
-    <t xml:space="preserve">exemple 1 </t>
-  </si>
-  <si>
-    <t>exemple 2</t>
-  </si>
-  <si>
-    <t>exemple 3</t>
-  </si>
-  <si>
-    <t>exemple 4</t>
-  </si>
-  <si>
-    <t>exemple 5</t>
-  </si>
-  <si>
-    <t>exemple 6</t>
+    <t>Brique 12</t>
+  </si>
+  <si>
+    <t>50 pieces</t>
+  </si>
+  <si>
+    <t>Brique 6</t>
+  </si>
+  <si>
+    <t>Ciment</t>
+  </si>
+  <si>
+    <t>5 Sac</t>
+  </si>
+  <si>
+    <t>lassaad</t>
+  </si>
+  <si>
+    <t>outillage</t>
+  </si>
+  <si>
+    <t>Sable</t>
+  </si>
+  <si>
+    <t>20 Pieces</t>
+  </si>
+  <si>
+    <t>meule a disque</t>
+  </si>
+  <si>
+    <t>réparation</t>
+  </si>
+  <si>
+    <t>Revetement Bar</t>
+  </si>
+  <si>
+    <t>11.34 m²</t>
+  </si>
+  <si>
+    <t>baguette rvt</t>
+  </si>
+  <si>
+    <t>2 unité</t>
+  </si>
+  <si>
+    <t>2 sac</t>
+  </si>
+  <si>
+    <t>ciment colle</t>
+  </si>
+  <si>
+    <t>Plomberie</t>
+  </si>
+  <si>
+    <t>PVC etc</t>
+  </si>
+  <si>
+    <t>Revetement toilette</t>
+  </si>
+  <si>
+    <t>22 m²</t>
+  </si>
+  <si>
+    <t>Sanitaire</t>
+  </si>
+  <si>
+    <t>4 urinoire + 4 robinet</t>
+  </si>
+  <si>
+    <t>barre 10</t>
+  </si>
+  <si>
+    <t>ciment blanc</t>
+  </si>
+  <si>
+    <t>disque diamon</t>
+  </si>
+  <si>
+    <t>fourniture elec</t>
+  </si>
+  <si>
+    <t>marbre comptoir</t>
+  </si>
+  <si>
+    <t>plomberie conduite</t>
+  </si>
+  <si>
+    <t>rmal</t>
+  </si>
+  <si>
+    <t>1 m3</t>
+  </si>
+  <si>
+    <t>disque diamond</t>
+  </si>
+  <si>
+    <t>location meule</t>
+  </si>
+  <si>
+    <t>reparation meule</t>
+  </si>
+  <si>
+    <t>sac vides</t>
+  </si>
+  <si>
+    <t>totalité payée</t>
+  </si>
+  <si>
+    <t>plomberie</t>
+  </si>
+  <si>
+    <t>rvt toilette</t>
+  </si>
+  <si>
+    <t>silicone</t>
+  </si>
+  <si>
+    <t>lumière wc</t>
+  </si>
+  <si>
+    <t>electricien</t>
+  </si>
+  <si>
+    <t>rchid</t>
+  </si>
+  <si>
+    <t>aide déplacement structure</t>
+  </si>
+  <si>
+    <t>électricité</t>
+  </si>
+  <si>
+    <t>panneau mdf</t>
+  </si>
+  <si>
+    <t>mahmoud rassaa</t>
+  </si>
+  <si>
+    <t>peinture</t>
+  </si>
+  <si>
+    <t>douilles</t>
+  </si>
+  <si>
+    <t>Naim</t>
+  </si>
+  <si>
+    <t>bache</t>
+  </si>
+  <si>
+    <t>divers</t>
+  </si>
+  <si>
+    <t>diver</t>
+  </si>
+  <si>
+    <t>adel</t>
   </si>
 </sst>
 </file>
@@ -309,9 +449,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -323,33 +463,39 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -362,22 +508,61 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF434343"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -400,11 +585,176 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -455,7 +805,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -478,16 +828,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -510,59 +860,100 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="11" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -700,23 +1091,23 @@
   </dxfs>
   <tableStyles count="3">
     <tableStyle name="suivi chantier-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="20"/>
-      <tableStyleElement type="headerRow" dxfId="19"/>
-      <tableStyleElement type="firstRowStripe" dxfId="18"/>
-      <tableStyleElement type="secondRowStripe" dxfId="17"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="14"/>
+      <tableStyleElement type="headerRow" dxfId="13"/>
+      <tableStyleElement type="firstRowStripe" dxfId="12"/>
+      <tableStyleElement type="secondRowStripe" dxfId="11"/>
     </tableStyle>
     <tableStyle name="estimation devis-style" pivot="0" count="5" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="16"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="totalRow" dxfId="14"/>
-      <tableStyleElement type="firstRowStripe" dxfId="13"/>
-      <tableStyleElement type="secondRowStripe" dxfId="12"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="10"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="secondRowStripe" dxfId="6"/>
     </tableStyle>
     <tableStyle name="Devis actuel-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="11"/>
-      <tableStyleElement type="headerRow" dxfId="10"/>
-      <tableStyleElement type="firstRowStripe" dxfId="9"/>
-      <tableStyleElement type="secondRowStripe" dxfId="8"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="5"/>
+      <tableStyleElement type="headerRow" dxfId="4"/>
+      <tableStyleElement type="firstRowStripe" dxfId="3"/>
+      <tableStyleElement type="secondRowStripe" dxfId="2"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -735,14 +1126,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:E7" headerRowDxfId="7" dataDxfId="6" totalsRowDxfId="5">
-  <autoFilter ref="A1:E7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:E65" headerRowDxfId="1" totalsRowDxfId="0">
+  <autoFilter ref="A1:E65" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Date" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nature" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Montant" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Commentaire" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Catégorie" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Date"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nature"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Montant"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Commentaire"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Catégorie"/>
   </tableColumns>
   <tableStyleInfo name="suivi chantier-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -981,7 +1372,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.42578125" customWidth="1"/>
@@ -992,7 +1383,7 @@
     <col min="7" max="7" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="22.5" customHeight="1">
+    <row r="1" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1009,943 +1400,1848 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="22.5" customHeight="1">
-      <c r="A2" s="51">
+    <row r="2" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A2" s="50">
         <v>46091</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="51" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="52">
+        <v>45</v>
+      </c>
+      <c r="D2" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="47">
+      <c r="E2" s="53" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A3" s="54">
+        <v>46091</v>
+      </c>
+      <c r="B3" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="56">
+        <v>80</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A4" s="58">
+        <v>46091</v>
+      </c>
+      <c r="B4" s="59" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="60">
+        <v>75</v>
+      </c>
+      <c r="D4" s="59" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A5" s="54">
+        <v>46091</v>
+      </c>
+      <c r="B5" s="62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="56">
+        <v>70</v>
+      </c>
+      <c r="D5" s="62" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A6" s="58">
+        <v>46091</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="60">
+        <v>120</v>
+      </c>
+      <c r="D6" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A7" s="54">
+        <v>46091</v>
+      </c>
+      <c r="B7" s="62" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="56">
         <v>400</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D7" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="48" t="s">
+      <c r="E7" s="57" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="22.5" customHeight="1">
-      <c r="A3" s="51">
+    <row r="8" spans="1:5" thickBot="1">
+      <c r="A8" s="58">
         <v>46091</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B8" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="60">
+        <v>86</v>
+      </c>
+      <c r="D8" s="63" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" thickBot="1">
+      <c r="A9" s="54">
+        <v>46091</v>
+      </c>
+      <c r="B9" s="62" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="56">
+        <v>50</v>
+      </c>
+      <c r="D9" s="62" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" thickBot="1">
+      <c r="A10" s="58">
+        <v>46092</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="60">
+        <v>17</v>
+      </c>
+      <c r="D10" s="59" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" thickBot="1">
+      <c r="A11" s="54">
+        <v>46092</v>
+      </c>
+      <c r="B11" s="55" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="47">
-        <f>76+10</f>
+      <c r="C11" s="64">
+        <v>14</v>
+      </c>
+      <c r="D11" s="55" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" thickBot="1">
+      <c r="A12" s="58">
+        <v>46092</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="60">
+        <v>30</v>
+      </c>
+      <c r="D12" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" thickBot="1">
+      <c r="A13" s="54">
+        <v>46092</v>
+      </c>
+      <c r="B13" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="56">
+        <v>504</v>
+      </c>
+      <c r="D13" s="62" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" thickBot="1">
+      <c r="A14" s="65">
+        <v>46093</v>
+      </c>
+      <c r="B14" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="60">
+        <v>17</v>
+      </c>
+      <c r="D14" s="63" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" thickBot="1">
+      <c r="A15" s="66">
+        <v>46093</v>
+      </c>
+      <c r="B15" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="56">
+        <v>30</v>
+      </c>
+      <c r="D15" s="62" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" thickBot="1">
+      <c r="A16" s="65">
+        <v>46093</v>
+      </c>
+      <c r="B16" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="60">
+        <v>22</v>
+      </c>
+      <c r="D16" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" thickBot="1">
+      <c r="A17" s="66">
+        <v>46093</v>
+      </c>
+      <c r="B17" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="56">
+        <v>65</v>
+      </c>
+      <c r="D17" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" thickBot="1">
+      <c r="A18" s="65">
+        <v>46093</v>
+      </c>
+      <c r="B18" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="60">
+        <v>200</v>
+      </c>
+      <c r="D18" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" thickBot="1">
+      <c r="A19" s="66">
+        <v>46093</v>
+      </c>
+      <c r="B19" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="56">
+        <v>200</v>
+      </c>
+      <c r="D19" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" thickBot="1">
+      <c r="A20" s="65">
+        <v>46093</v>
+      </c>
+      <c r="B20" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="60">
+        <v>40</v>
+      </c>
+      <c r="D20" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30.75" thickBot="1">
+      <c r="A21" s="66">
+        <v>46093</v>
+      </c>
+      <c r="B21" s="55" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="56">
+        <v>418</v>
+      </c>
+      <c r="D21" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="27" thickBot="1">
+      <c r="A22" s="65">
+        <v>46093</v>
+      </c>
+      <c r="B22" s="59" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="60">
+        <v>981</v>
+      </c>
+      <c r="D22" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="E22" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" thickBot="1">
+      <c r="A23" s="66">
+        <v>46095</v>
+      </c>
+      <c r="B23" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="D3" s="46" t="s">
+      <c r="C23" s="56">
+        <v>20</v>
+      </c>
+      <c r="D23" s="67"/>
+      <c r="E23" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" thickBot="1">
+      <c r="A24" s="65">
+        <v>46095</v>
+      </c>
+      <c r="B24" s="59" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="60">
+        <v>20</v>
+      </c>
+      <c r="D24" s="68"/>
+      <c r="E24" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" thickBot="1">
+      <c r="A25" s="66">
+        <v>46095</v>
+      </c>
+      <c r="B25" s="55" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="56">
+        <v>20</v>
+      </c>
+      <c r="D25" s="67"/>
+      <c r="E25" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" thickBot="1">
+      <c r="A26" s="65">
+        <v>46095</v>
+      </c>
+      <c r="B26" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" s="60">
+        <v>27</v>
+      </c>
+      <c r="D26" s="68"/>
+      <c r="E26" s="61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" thickBot="1">
+      <c r="A27" s="66">
+        <v>46095</v>
+      </c>
+      <c r="B27" s="55" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="56">
+        <v>110</v>
+      </c>
+      <c r="D27" s="67"/>
+      <c r="E27" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" thickBot="1">
+      <c r="A28" s="65">
+        <v>46095</v>
+      </c>
+      <c r="B28" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="60">
+        <v>140</v>
+      </c>
+      <c r="D28" s="68"/>
+      <c r="E28" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" thickBot="1">
+      <c r="A29" s="66">
+        <v>46095</v>
+      </c>
+      <c r="B29" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="56">
+        <v>500</v>
+      </c>
+      <c r="D29" s="67"/>
+      <c r="E29" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" thickBot="1">
+      <c r="A30" s="65">
+        <v>46095</v>
+      </c>
+      <c r="B30" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="60">
+        <v>120</v>
+      </c>
+      <c r="D30" s="68"/>
+      <c r="E30" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="30.75" thickBot="1">
+      <c r="A31" s="66">
+        <v>46095</v>
+      </c>
+      <c r="B31" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="56">
+        <v>200</v>
+      </c>
+      <c r="D31" s="67"/>
+      <c r="E31" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" thickBot="1">
+      <c r="A32" s="65">
+        <v>46095</v>
+      </c>
+      <c r="B32" s="59" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" s="60">
+        <v>60</v>
+      </c>
+      <c r="D32" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="E32" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" thickBot="1">
+      <c r="A33" s="66">
+        <v>46096</v>
+      </c>
+      <c r="B33" s="55" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="56">
+        <v>16</v>
+      </c>
+      <c r="D33" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="57" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" thickBot="1">
+      <c r="A34" s="65">
+        <v>46097</v>
+      </c>
+      <c r="B34" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="60">
+        <v>20</v>
+      </c>
+      <c r="D34" s="68"/>
+      <c r="E34" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" thickBot="1">
+      <c r="A35" s="66">
+        <v>46097</v>
+      </c>
+      <c r="B35" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="56">
+        <v>200</v>
+      </c>
+      <c r="D35" s="67"/>
+      <c r="E35" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" thickBot="1">
+      <c r="A36" s="65">
+        <v>46098</v>
+      </c>
+      <c r="B36" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" s="60">
+        <v>8.5</v>
+      </c>
+      <c r="D36" s="68"/>
+      <c r="E36" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" thickBot="1">
+      <c r="A37" s="66">
+        <v>46099</v>
+      </c>
+      <c r="B37" s="55" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="56">
+        <v>8</v>
+      </c>
+      <c r="D37" s="67"/>
+      <c r="E37" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" thickBot="1">
+      <c r="A38" s="65">
+        <v>46099</v>
+      </c>
+      <c r="B38" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="60">
+        <v>8</v>
+      </c>
+      <c r="D38" s="68"/>
+      <c r="E38" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" thickBot="1">
+      <c r="A39" s="66">
+        <v>46099</v>
+      </c>
+      <c r="B39" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="56">
+        <v>50</v>
+      </c>
+      <c r="D39" s="67"/>
+      <c r="E39" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" thickBot="1">
+      <c r="A40" s="65">
+        <v>46099</v>
+      </c>
+      <c r="B40" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="C40" s="60">
+        <v>15</v>
+      </c>
+      <c r="D40" s="68"/>
+      <c r="E40" s="61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" thickBot="1">
+      <c r="A41" s="66">
+        <v>46099</v>
+      </c>
+      <c r="B41" s="55" t="s">
+        <v>96</v>
+      </c>
+      <c r="C41" s="56">
+        <v>10</v>
+      </c>
+      <c r="D41" s="67"/>
+      <c r="E41" s="57" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" thickBot="1">
+      <c r="A42" s="65">
+        <v>46099</v>
+      </c>
+      <c r="B42" s="59" t="s">
+        <v>97</v>
+      </c>
+      <c r="C42" s="60">
+        <v>6</v>
+      </c>
+      <c r="D42" s="68"/>
+      <c r="E42" s="61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" thickBot="1">
+      <c r="A43" s="66">
+        <v>46100</v>
+      </c>
+      <c r="B43" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C43" s="56">
+        <v>350</v>
+      </c>
+      <c r="D43" s="62" t="s">
+        <v>98</v>
+      </c>
+      <c r="E43" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" thickBot="1">
+      <c r="A44" s="65">
+        <v>46100</v>
+      </c>
+      <c r="B44" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="60">
+        <v>110</v>
+      </c>
+      <c r="D44" s="68"/>
+      <c r="E44" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" thickBot="1">
+      <c r="A45" s="66">
+        <v>46100</v>
+      </c>
+      <c r="B45" s="55" t="s">
+        <v>100</v>
+      </c>
+      <c r="C45" s="56">
+        <v>38</v>
+      </c>
+      <c r="D45" s="67"/>
+      <c r="E45" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" thickBot="1">
+      <c r="A46" s="65">
+        <v>46100</v>
+      </c>
+      <c r="B46" s="59" t="s">
+        <v>101</v>
+      </c>
+      <c r="C46" s="60">
+        <v>11</v>
+      </c>
+      <c r="D46" s="68"/>
+      <c r="E46" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" thickBot="1">
+      <c r="A47" s="66">
+        <v>46100</v>
+      </c>
+      <c r="B47" s="55" t="s">
+        <v>102</v>
+      </c>
+      <c r="C47" s="56">
+        <v>10</v>
+      </c>
+      <c r="D47" s="67"/>
+      <c r="E47" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" thickBot="1">
+      <c r="A48" s="65">
+        <v>46100</v>
+      </c>
+      <c r="B48" s="59" t="s">
+        <v>103</v>
+      </c>
+      <c r="C48" s="60">
+        <v>10</v>
+      </c>
+      <c r="D48" s="68"/>
+      <c r="E48" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="27" thickBot="1">
+      <c r="A49" s="66">
+        <v>46103</v>
+      </c>
+      <c r="B49" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" s="56">
+        <v>20</v>
+      </c>
+      <c r="D49" s="62" t="s">
+        <v>105</v>
+      </c>
+      <c r="E49" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" thickBot="1">
+      <c r="A50" s="65">
+        <v>46104</v>
+      </c>
+      <c r="B50" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" s="60">
+        <v>120</v>
+      </c>
+      <c r="D50" s="63" t="s">
+        <v>98</v>
+      </c>
+      <c r="E50" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" thickBot="1">
+      <c r="A51" s="66">
+        <v>46104</v>
+      </c>
+      <c r="B51" s="55" t="s">
+        <v>106</v>
+      </c>
+      <c r="C51" s="56">
+        <v>200</v>
+      </c>
+      <c r="D51" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="E51" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" thickBot="1">
+      <c r="A52" s="65">
+        <v>46109</v>
+      </c>
+      <c r="B52" s="59" t="s">
+        <v>107</v>
+      </c>
+      <c r="C52" s="60">
+        <v>277</v>
+      </c>
+      <c r="D52" s="68"/>
+      <c r="E52" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" thickBot="1">
+      <c r="A53" s="66">
+        <v>46113</v>
+      </c>
+      <c r="B53" s="55" t="s">
+        <v>108</v>
+      </c>
+      <c r="C53" s="56">
+        <v>130</v>
+      </c>
+      <c r="D53" s="67"/>
+      <c r="E53" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" thickBot="1">
+      <c r="A54" s="65">
+        <v>46117</v>
+      </c>
+      <c r="B54" s="59" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" s="60">
+        <v>15</v>
+      </c>
+      <c r="D54" s="68"/>
+      <c r="E54" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" thickBot="1">
+      <c r="A55" s="66">
+        <v>46117</v>
+      </c>
+      <c r="B55" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" s="56">
         <v>7</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="D55" s="67"/>
+      <c r="E55" s="57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" thickBot="1">
+      <c r="A56" s="65">
+        <v>46117</v>
+      </c>
+      <c r="B56" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="C56" s="60">
+        <v>50</v>
+      </c>
+      <c r="D56" s="68"/>
+      <c r="E56" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" thickBot="1">
+      <c r="A57" s="66">
+        <v>46120</v>
+      </c>
+      <c r="B57" s="55" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" s="56">
+        <v>160</v>
+      </c>
+      <c r="D57" s="67"/>
+      <c r="E57" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" thickBot="1">
+      <c r="A58" s="65">
+        <v>46120</v>
+      </c>
+      <c r="B58" s="59" t="s">
+        <v>110</v>
+      </c>
+      <c r="C58" s="60">
+        <v>10</v>
+      </c>
+      <c r="D58" s="68"/>
+      <c r="E58" s="61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" thickBot="1">
+      <c r="A59" s="66">
+        <v>46122</v>
+      </c>
+      <c r="B59" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="C59" s="56">
+        <v>500</v>
+      </c>
+      <c r="D59" s="67"/>
+      <c r="E59" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" thickBot="1">
+      <c r="A60" s="65">
+        <v>46122</v>
+      </c>
+      <c r="B60" s="59" t="s">
+        <v>111</v>
+      </c>
+      <c r="C60" s="60">
+        <v>370</v>
+      </c>
+      <c r="D60" s="68"/>
+      <c r="E60" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" thickBot="1">
+      <c r="A61" s="66">
+        <v>46122</v>
+      </c>
+      <c r="B61" s="55" t="s">
+        <v>112</v>
+      </c>
+      <c r="C61" s="56">
+        <v>10</v>
+      </c>
+      <c r="D61" s="67"/>
+      <c r="E61" s="57" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="22.5" customHeight="1">
-      <c r="A4" s="51">
-        <v>46091</v>
-      </c>
-      <c r="B4" s="46" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" s="47">
-        <v>70</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="48" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="22.5" customHeight="1">
-      <c r="A5" s="51">
-        <v>46091</v>
-      </c>
-      <c r="B5" s="46" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="47">
+    <row r="62" spans="1:5" thickBot="1">
+      <c r="A62" s="65">
+        <v>46123</v>
+      </c>
+      <c r="B62" s="59" t="s">
+        <v>113</v>
+      </c>
+      <c r="C62" s="60">
+        <v>60</v>
+      </c>
+      <c r="D62" s="68"/>
+      <c r="E62" s="61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" thickBot="1">
+      <c r="A63" s="66">
+        <v>46124</v>
+      </c>
+      <c r="B63" s="55" t="s">
+        <v>114</v>
+      </c>
+      <c r="C63" s="56">
+        <v>26</v>
+      </c>
+      <c r="D63" s="67"/>
+      <c r="E63" s="57" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" thickBot="1">
+      <c r="A64" s="65">
+        <v>46124</v>
+      </c>
+      <c r="B64" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="C64" s="60">
         <v>50</v>
       </c>
-      <c r="D5" s="46" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="48" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="22.5" customHeight="1">
-      <c r="A6" s="51">
-        <v>46091</v>
-      </c>
-      <c r="B6" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="47">
-        <v>75</v>
-      </c>
-      <c r="D6" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="48" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="22.5" customHeight="1">
-      <c r="A7" s="51">
-        <v>46091</v>
-      </c>
-      <c r="B7" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="47">
-        <v>80</v>
-      </c>
-      <c r="D7" s="48" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="48" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="12.75">
-      <c r="A8" s="52"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" ht="12.75">
-      <c r="A9" s="52"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" ht="12.75">
-      <c r="A10" s="52"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" ht="12.75">
-      <c r="A11" s="52"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" ht="12.75">
-      <c r="A12" s="52"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" ht="12.75">
-      <c r="A13" s="52"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" ht="12.75">
-      <c r="A14" s="52"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" ht="12.75">
-      <c r="A15" s="52"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" ht="12.75">
-      <c r="A16" s="52"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="1:5" ht="12.75">
-      <c r="A17" s="52"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:5" ht="12.75">
-      <c r="A18" s="52"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:5" ht="12.75">
-      <c r="A19" s="52"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:5" ht="12.75">
-      <c r="A20" s="52"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" ht="12.75">
-      <c r="A21" s="52"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:5" ht="12.75">
-      <c r="A22" s="52"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" ht="12.75">
-      <c r="A23" s="52"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="12.75">
-      <c r="A24" s="52"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-    </row>
-    <row r="25" spans="1:5" ht="12.75">
-      <c r="A25" s="52"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-    </row>
-    <row r="26" spans="1:5" ht="12.75">
-      <c r="A26" s="52"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" ht="12.75">
-      <c r="A27" s="52"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="1:5" ht="12.75">
-      <c r="A28" s="52"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-    </row>
-    <row r="29" spans="1:5" ht="12.75">
-      <c r="A29" s="52"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-    </row>
-    <row r="30" spans="1:5" ht="12.75">
-      <c r="A30" s="52"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-    </row>
-    <row r="31" spans="1:5" ht="12.75">
-      <c r="A31" s="52"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-    </row>
-    <row r="32" spans="1:5" ht="12.75">
-      <c r="A32" s="52"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-    </row>
-    <row r="33" spans="1:5" ht="12.75">
-      <c r="A33" s="52"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="1:5" ht="12.75">
-      <c r="A34" s="52"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-    </row>
-    <row r="35" spans="1:5" ht="12.75">
-      <c r="A35" s="52"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-    </row>
-    <row r="36" spans="1:5" ht="12.75">
-      <c r="A36" s="52"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
-    </row>
-    <row r="37" spans="1:5" ht="12.75">
-      <c r="A37" s="52"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-    </row>
-    <row r="38" spans="1:5" ht="12.75">
-      <c r="A38" s="52"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-    </row>
-    <row r="39" spans="1:5" ht="12.75">
-      <c r="A39" s="52"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-    </row>
-    <row r="40" spans="1:5" ht="12.75">
-      <c r="A40" s="52"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-    </row>
-    <row r="41" spans="1:5" ht="12.75">
-      <c r="A41" s="52"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-    </row>
-    <row r="42" spans="1:5" ht="12.75">
-      <c r="A42" s="52"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-    </row>
-    <row r="43" spans="1:5" ht="12.75">
-      <c r="A43" s="52"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-    </row>
-    <row r="44" spans="1:5" ht="12.75">
-      <c r="A44" s="52"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-    </row>
-    <row r="45" spans="1:5" ht="12.75">
-      <c r="A45" s="52"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-    </row>
-    <row r="46" spans="1:5" ht="12.75">
-      <c r="A46" s="52"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-    </row>
-    <row r="47" spans="1:5" ht="12.75">
-      <c r="A47" s="52"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-    </row>
-    <row r="48" spans="1:5" ht="12.75">
-      <c r="A48" s="52"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-    </row>
-    <row r="49" spans="1:5" ht="12.75">
-      <c r="A49" s="52"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-    </row>
-    <row r="50" spans="1:5" ht="12.75">
-      <c r="A50" s="52"/>
-      <c r="B50" s="1"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-    </row>
-    <row r="51" spans="1:5" ht="12.75">
-      <c r="A51" s="52"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
-    </row>
-    <row r="52" spans="1:5" ht="12.75">
-      <c r="A52" s="52"/>
-      <c r="B52" s="1"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="1"/>
-      <c r="E52" s="1"/>
-    </row>
-    <row r="53" spans="1:5" ht="12.75">
-      <c r="A53" s="52"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-    </row>
-    <row r="54" spans="1:5" ht="12.75">
-      <c r="A54" s="52"/>
-      <c r="B54" s="1"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-    </row>
-    <row r="55" spans="1:5" ht="12.75">
-      <c r="A55" s="52"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-    </row>
-    <row r="56" spans="1:5" ht="12.75">
-      <c r="A56" s="52"/>
-      <c r="B56" s="1"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
-    </row>
-    <row r="57" spans="1:5" ht="12.75">
-      <c r="A57" s="52"/>
-      <c r="B57" s="1"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
-    </row>
-    <row r="58" spans="1:5" ht="12.75">
-      <c r="A58" s="52"/>
-      <c r="B58" s="1"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
-    </row>
-    <row r="59" spans="1:5" ht="12.75">
-      <c r="A59" s="52"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-    </row>
-    <row r="60" spans="1:5" ht="12.75">
-      <c r="A60" s="52"/>
-      <c r="B60" s="1"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-    </row>
-    <row r="61" spans="1:5" ht="12.75">
-      <c r="A61" s="52"/>
-      <c r="B61" s="1"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
-    </row>
-    <row r="62" spans="1:5" ht="12.75">
-      <c r="A62" s="52"/>
-      <c r="B62" s="1"/>
-      <c r="C62" s="4"/>
-      <c r="D62" s="1"/>
-      <c r="E62" s="1"/>
-    </row>
-    <row r="63" spans="1:5" ht="12.75">
-      <c r="A63" s="52"/>
-      <c r="B63" s="1"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="1"/>
-      <c r="E63" s="1"/>
-    </row>
-    <row r="64" spans="1:5" ht="12.75">
-      <c r="A64" s="52"/>
-      <c r="B64" s="1"/>
-      <c r="C64" s="4"/>
-      <c r="D64" s="1"/>
-      <c r="E64" s="1"/>
-    </row>
-    <row r="65" spans="1:5" ht="12.75">
-      <c r="A65" s="52"/>
-      <c r="B65" s="1"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="1"/>
-      <c r="E65" s="1"/>
+      <c r="D64" s="68"/>
+      <c r="E64" s="61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" thickBot="1">
+      <c r="A65" s="69">
+        <v>46124</v>
+      </c>
+      <c r="B65" s="70" t="s">
+        <v>115</v>
+      </c>
+      <c r="C65" s="71">
+        <v>40</v>
+      </c>
+      <c r="D65" s="72"/>
+      <c r="E65" s="73" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="66" spans="1:5" ht="12.75">
-      <c r="A66" s="52"/>
+      <c r="A66" s="46"/>
       <c r="B66" s="1"/>
       <c r="C66" s="4"/>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
     </row>
     <row r="67" spans="1:5" ht="12.75">
-      <c r="A67" s="52"/>
+      <c r="A67" s="46"/>
       <c r="B67" s="1"/>
       <c r="C67" s="4"/>
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
     </row>
     <row r="68" spans="1:5" ht="12.75">
-      <c r="A68" s="52"/>
+      <c r="A68" s="46"/>
       <c r="B68" s="1"/>
       <c r="C68" s="4"/>
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
     </row>
     <row r="69" spans="1:5" ht="12.75">
-      <c r="A69" s="52"/>
+      <c r="A69" s="46"/>
       <c r="B69" s="1"/>
       <c r="C69" s="4"/>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
     </row>
     <row r="70" spans="1:5" ht="12.75">
-      <c r="A70" s="52"/>
+      <c r="A70" s="46"/>
       <c r="B70" s="1"/>
       <c r="C70" s="4"/>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
     </row>
     <row r="71" spans="1:5" ht="12.75">
-      <c r="A71" s="53"/>
+      <c r="A71" s="46"/>
+      <c r="B71" s="1"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
     </row>
     <row r="72" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A72" s="53"/>
+      <c r="A72" s="46"/>
+      <c r="B72" s="1"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
     </row>
     <row r="73" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A73" s="53"/>
+      <c r="A73" s="46"/>
+      <c r="B73" s="1"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
     </row>
     <row r="74" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A74" s="53"/>
+      <c r="A74" s="46"/>
+      <c r="B74" s="1"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
     </row>
     <row r="75" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A75" s="53"/>
+      <c r="A75" s="46"/>
+      <c r="B75" s="1"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
     </row>
     <row r="76" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A76" s="53"/>
+      <c r="A76" s="46"/>
+      <c r="B76" s="1"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
     </row>
     <row r="77" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A77" s="53"/>
+      <c r="A77" s="46"/>
+      <c r="B77" s="1"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
     </row>
     <row r="78" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A78" s="53"/>
+      <c r="A78" s="46"/>
+      <c r="B78" s="1"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="1"/>
+      <c r="E78" s="1"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A79" s="53"/>
+      <c r="A79" s="46"/>
+      <c r="B79" s="1"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
     </row>
     <row r="80" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A80" s="53"/>
-    </row>
-    <row r="81" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A81" s="53"/>
-    </row>
-    <row r="82" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A82" s="53"/>
-    </row>
-    <row r="83" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A83" s="53"/>
-    </row>
-    <row r="84" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A84" s="53"/>
-    </row>
-    <row r="85" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A85" s="53"/>
-    </row>
-    <row r="86" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A86" s="53"/>
-    </row>
-    <row r="87" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A87" s="53"/>
-    </row>
-    <row r="88" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A88" s="53"/>
-    </row>
-    <row r="89" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A89" s="53"/>
-    </row>
-    <row r="90" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A90" s="53"/>
-    </row>
-    <row r="91" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A91" s="53"/>
-    </row>
-    <row r="92" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A92" s="53"/>
-    </row>
-    <row r="93" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A93" s="53"/>
-    </row>
-    <row r="94" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A94" s="53"/>
-    </row>
-    <row r="95" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A95" s="53"/>
-    </row>
-    <row r="96" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A96" s="53"/>
-    </row>
-    <row r="97" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A97" s="53"/>
-    </row>
-    <row r="98" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A98" s="53"/>
-    </row>
-    <row r="99" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A99" s="53"/>
-    </row>
-    <row r="100" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A100" s="53"/>
-    </row>
-    <row r="101" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A101" s="53"/>
-    </row>
-    <row r="102" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A102" s="53"/>
-    </row>
-    <row r="103" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A103" s="53"/>
-    </row>
-    <row r="104" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A104" s="53"/>
-    </row>
-    <row r="105" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A105" s="53"/>
-    </row>
-    <row r="106" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A106" s="53"/>
-    </row>
-    <row r="107" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A107" s="53"/>
-    </row>
-    <row r="108" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A108" s="53"/>
-    </row>
-    <row r="109" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A109" s="53"/>
-    </row>
-    <row r="110" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A110" s="53"/>
-    </row>
-    <row r="111" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A111" s="53"/>
-    </row>
-    <row r="112" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A112" s="53"/>
-    </row>
-    <row r="113" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A113" s="53"/>
-    </row>
-    <row r="114" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A114" s="53"/>
-    </row>
-    <row r="115" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A115" s="53"/>
-    </row>
-    <row r="116" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A116" s="53"/>
-    </row>
-    <row r="117" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A117" s="53"/>
-    </row>
-    <row r="118" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A118" s="53"/>
-    </row>
-    <row r="119" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A119" s="53"/>
-    </row>
-    <row r="120" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A120" s="53"/>
-    </row>
-    <row r="121" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A121" s="53"/>
-    </row>
-    <row r="122" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A122" s="53"/>
-    </row>
-    <row r="123" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A123" s="53"/>
-    </row>
-    <row r="124" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A124" s="53"/>
-    </row>
-    <row r="125" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A125" s="53"/>
-    </row>
-    <row r="126" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A126" s="53"/>
-    </row>
-    <row r="127" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A127" s="53"/>
-    </row>
-    <row r="128" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A128" s="53"/>
+      <c r="A80" s="46"/>
+      <c r="B80" s="1"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="1"/>
+      <c r="E80" s="1"/>
+    </row>
+    <row r="81" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A81" s="46"/>
+      <c r="B81" s="1"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="1"/>
+      <c r="E81" s="1"/>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A82" s="46"/>
+      <c r="B82" s="1"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="1"/>
+    </row>
+    <row r="83" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A83" s="46"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
+    </row>
+    <row r="84" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A84" s="46"/>
+      <c r="B84" s="1"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="1"/>
+    </row>
+    <row r="85" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A85" s="46"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="1"/>
+    </row>
+    <row r="86" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A86" s="46"/>
+      <c r="B86" s="1"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+    </row>
+    <row r="87" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A87" s="46"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A88" s="46"/>
+      <c r="B88" s="1"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A89" s="46"/>
+      <c r="B89" s="1"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+    </row>
+    <row r="90" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A90" s="46"/>
+      <c r="B90" s="1"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+    </row>
+    <row r="91" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A91" s="46"/>
+      <c r="B91" s="1"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+    </row>
+    <row r="92" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A92" s="46"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+    </row>
+    <row r="93" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A93" s="46"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+    </row>
+    <row r="94" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A94" s="46"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+    </row>
+    <row r="95" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A95" s="46"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+    </row>
+    <row r="96" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A96" s="46"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="4"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+    </row>
+    <row r="97" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A97" s="46"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+    </row>
+    <row r="98" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A98" s="46"/>
+      <c r="B98" s="1"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+    </row>
+    <row r="99" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A99" s="46"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+    </row>
+    <row r="100" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A100" s="46"/>
+      <c r="B100" s="1"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+    </row>
+    <row r="101" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A101" s="46"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+    </row>
+    <row r="102" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A102" s="46"/>
+      <c r="B102" s="1"/>
+      <c r="C102" s="4"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+    </row>
+    <row r="103" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A103" s="46"/>
+      <c r="B103" s="1"/>
+      <c r="C103" s="4"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+    </row>
+    <row r="104" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A104" s="46"/>
+      <c r="B104" s="1"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+    </row>
+    <row r="105" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A105" s="46"/>
+      <c r="B105" s="1"/>
+      <c r="C105" s="4"/>
+      <c r="D105" s="1"/>
+      <c r="E105" s="1"/>
+    </row>
+    <row r="106" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A106" s="46"/>
+      <c r="B106" s="1"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+    </row>
+    <row r="107" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A107" s="46"/>
+      <c r="B107" s="1"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="1"/>
+      <c r="E107" s="1"/>
+    </row>
+    <row r="108" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A108" s="46"/>
+      <c r="B108" s="1"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="1"/>
+      <c r="E108" s="1"/>
+    </row>
+    <row r="109" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A109" s="46"/>
+      <c r="B109" s="1"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="1"/>
+      <c r="E109" s="1"/>
+    </row>
+    <row r="110" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A110" s="46"/>
+      <c r="B110" s="1"/>
+      <c r="C110" s="4"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+    </row>
+    <row r="111" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A111" s="46"/>
+      <c r="B111" s="1"/>
+      <c r="C111" s="4"/>
+      <c r="D111" s="1"/>
+      <c r="E111" s="1"/>
+    </row>
+    <row r="112" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A112" s="46"/>
+      <c r="B112" s="1"/>
+      <c r="C112" s="4"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+    </row>
+    <row r="113" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A113" s="46"/>
+      <c r="B113" s="1"/>
+      <c r="C113" s="4"/>
+      <c r="D113" s="1"/>
+      <c r="E113" s="1"/>
+    </row>
+    <row r="114" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A114" s="46"/>
+      <c r="B114" s="1"/>
+      <c r="C114" s="4"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
+    </row>
+    <row r="115" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A115" s="46"/>
+      <c r="B115" s="1"/>
+      <c r="C115" s="4"/>
+      <c r="D115" s="1"/>
+      <c r="E115" s="1"/>
+    </row>
+    <row r="116" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A116" s="46"/>
+      <c r="B116" s="1"/>
+      <c r="C116" s="4"/>
+      <c r="D116" s="1"/>
+      <c r="E116" s="1"/>
+    </row>
+    <row r="117" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A117" s="46"/>
+      <c r="B117" s="1"/>
+      <c r="C117" s="4"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="1"/>
+    </row>
+    <row r="118" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A118" s="46"/>
+      <c r="B118" s="1"/>
+      <c r="C118" s="4"/>
+      <c r="D118" s="1"/>
+      <c r="E118" s="1"/>
+    </row>
+    <row r="119" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A119" s="46"/>
+      <c r="B119" s="1"/>
+      <c r="C119" s="4"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="1"/>
+    </row>
+    <row r="120" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A120" s="46"/>
+      <c r="B120" s="1"/>
+      <c r="C120" s="4"/>
+      <c r="D120" s="1"/>
+      <c r="E120" s="1"/>
+    </row>
+    <row r="121" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A121" s="46"/>
+      <c r="B121" s="1"/>
+      <c r="C121" s="4"/>
+      <c r="D121" s="1"/>
+      <c r="E121" s="1"/>
+    </row>
+    <row r="122" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A122" s="46"/>
+      <c r="B122" s="1"/>
+      <c r="C122" s="4"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="1"/>
+    </row>
+    <row r="123" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A123" s="46"/>
+      <c r="B123" s="1"/>
+      <c r="C123" s="4"/>
+      <c r="D123" s="1"/>
+      <c r="E123" s="1"/>
+    </row>
+    <row r="124" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A124" s="46"/>
+      <c r="B124" s="1"/>
+      <c r="C124" s="4"/>
+      <c r="D124" s="1"/>
+      <c r="E124" s="1"/>
+    </row>
+    <row r="125" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A125" s="46"/>
+      <c r="B125" s="1"/>
+      <c r="C125" s="4"/>
+      <c r="D125" s="1"/>
+      <c r="E125" s="1"/>
+    </row>
+    <row r="126" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A126" s="46"/>
+      <c r="B126" s="1"/>
+      <c r="C126" s="4"/>
+      <c r="D126" s="1"/>
+      <c r="E126" s="1"/>
+    </row>
+    <row r="127" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A127" s="46"/>
+      <c r="B127" s="1"/>
+      <c r="C127" s="4"/>
+      <c r="D127" s="1"/>
+      <c r="E127" s="1"/>
+    </row>
+    <row r="128" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A128" s="46"/>
+      <c r="B128" s="1"/>
+      <c r="C128" s="4"/>
+      <c r="D128" s="1"/>
+      <c r="E128" s="1"/>
     </row>
     <row r="129" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A129" s="53"/>
+      <c r="A129" s="47"/>
     </row>
     <row r="130" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A130" s="53"/>
+      <c r="A130" s="47"/>
     </row>
     <row r="131" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A131" s="53"/>
+      <c r="A131" s="47"/>
     </row>
     <row r="132" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A132" s="53"/>
+      <c r="A132" s="47"/>
     </row>
     <row r="133" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A133" s="53"/>
+      <c r="A133" s="47"/>
     </row>
     <row r="134" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A134" s="53"/>
+      <c r="A134" s="47"/>
     </row>
     <row r="135" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A135" s="53"/>
+      <c r="A135" s="47"/>
     </row>
     <row r="136" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A136" s="53"/>
+      <c r="A136" s="47"/>
     </row>
     <row r="137" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A137" s="53"/>
+      <c r="A137" s="47"/>
     </row>
     <row r="138" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A138" s="53"/>
+      <c r="A138" s="47"/>
     </row>
     <row r="139" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A139" s="53"/>
+      <c r="A139" s="47"/>
     </row>
     <row r="140" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A140" s="53"/>
+      <c r="A140" s="47"/>
     </row>
     <row r="141" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A141" s="53"/>
+      <c r="A141" s="47"/>
     </row>
     <row r="142" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A142" s="53"/>
+      <c r="A142" s="47"/>
     </row>
     <row r="143" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A143" s="53"/>
+      <c r="A143" s="47"/>
     </row>
     <row r="144" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A144" s="53"/>
+      <c r="A144" s="47"/>
     </row>
     <row r="145" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A145" s="53"/>
+      <c r="A145" s="47"/>
     </row>
     <row r="146" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A146" s="53"/>
+      <c r="A146" s="47"/>
     </row>
     <row r="147" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A147" s="53"/>
+      <c r="A147" s="47"/>
     </row>
     <row r="148" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A148" s="53"/>
+      <c r="A148" s="47"/>
     </row>
     <row r="149" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A149" s="53"/>
+      <c r="A149" s="47"/>
     </row>
     <row r="150" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A150" s="53"/>
+      <c r="A150" s="47"/>
     </row>
     <row r="151" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A151" s="53"/>
+      <c r="A151" s="47"/>
     </row>
     <row r="152" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A152" s="53"/>
+      <c r="A152" s="47"/>
     </row>
     <row r="153" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A153" s="53"/>
+      <c r="A153" s="47"/>
     </row>
     <row r="154" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A154" s="53"/>
+      <c r="A154" s="47"/>
     </row>
     <row r="155" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A155" s="53"/>
+      <c r="A155" s="47"/>
     </row>
     <row r="156" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A156" s="53"/>
+      <c r="A156" s="47"/>
     </row>
     <row r="157" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A157" s="53"/>
+      <c r="A157" s="47"/>
     </row>
     <row r="158" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A158" s="53"/>
+      <c r="A158" s="47"/>
     </row>
     <row r="159" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A159" s="53"/>
+      <c r="A159" s="47"/>
     </row>
     <row r="160" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A160" s="53"/>
+      <c r="A160" s="47"/>
     </row>
     <row r="161" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A161" s="53"/>
+      <c r="A161" s="47"/>
     </row>
     <row r="162" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A162" s="53"/>
+      <c r="A162" s="47"/>
     </row>
     <row r="163" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A163" s="53"/>
+      <c r="A163" s="47"/>
     </row>
     <row r="164" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A164" s="53"/>
+      <c r="A164" s="47"/>
     </row>
     <row r="165" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A165" s="53"/>
+      <c r="A165" s="47"/>
     </row>
     <row r="166" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A166" s="53"/>
+      <c r="A166" s="47"/>
     </row>
     <row r="167" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A167" s="53"/>
+      <c r="A167" s="47"/>
     </row>
     <row r="168" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A168" s="53"/>
+      <c r="A168" s="47"/>
     </row>
     <row r="169" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A169" s="53"/>
+      <c r="A169" s="47"/>
     </row>
     <row r="170" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A170" s="53"/>
+      <c r="A170" s="47"/>
     </row>
     <row r="171" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A171" s="53"/>
+      <c r="A171" s="47"/>
     </row>
     <row r="172" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A172" s="53"/>
+      <c r="A172" s="47"/>
     </row>
     <row r="173" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A173" s="53"/>
+      <c r="A173" s="47"/>
     </row>
     <row r="174" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A174" s="53"/>
+      <c r="A174" s="47"/>
     </row>
     <row r="175" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A175" s="53"/>
+      <c r="A175" s="47"/>
     </row>
     <row r="176" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A176" s="53"/>
+      <c r="A176" s="47"/>
     </row>
     <row r="177" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A177" s="53"/>
+      <c r="A177" s="47"/>
     </row>
     <row r="178" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A178" s="53"/>
+      <c r="A178" s="47"/>
     </row>
     <row r="179" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A179" s="53"/>
+      <c r="A179" s="47"/>
     </row>
     <row r="180" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A180" s="53"/>
+      <c r="A180" s="47"/>
     </row>
     <row r="181" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A181" s="53"/>
+      <c r="A181" s="47"/>
     </row>
     <row r="182" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A182" s="53"/>
+      <c r="A182" s="47"/>
     </row>
     <row r="183" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A183" s="53"/>
+      <c r="A183" s="47"/>
     </row>
     <row r="184" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A184" s="53"/>
+      <c r="A184" s="47"/>
     </row>
     <row r="185" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A185" s="53"/>
+      <c r="A185" s="47"/>
     </row>
     <row r="186" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A186" s="53"/>
+      <c r="A186" s="47"/>
     </row>
     <row r="187" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A187" s="53"/>
+      <c r="A187" s="47"/>
     </row>
     <row r="188" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A188" s="53"/>
+      <c r="A188" s="47"/>
     </row>
     <row r="189" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A189" s="53"/>
+      <c r="A189" s="47"/>
     </row>
     <row r="190" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A190" s="53"/>
+      <c r="A190" s="47"/>
     </row>
     <row r="191" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A191" s="53"/>
+      <c r="A191" s="47"/>
     </row>
     <row r="192" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A192" s="53"/>
+      <c r="A192" s="47"/>
     </row>
     <row r="193" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A193" s="53"/>
+      <c r="A193" s="47"/>
+    </row>
+    <row r="194" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A194" s="47"/>
+    </row>
+    <row r="195" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A195" s="47"/>
+    </row>
+    <row r="196" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A196" s="47"/>
+    </row>
+    <row r="197" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A197" s="47"/>
+    </row>
+    <row r="198" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A198" s="47"/>
+    </row>
+    <row r="199" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A199" s="47"/>
+    </row>
+    <row r="200" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A200" s="47"/>
+    </row>
+    <row r="201" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A201" s="47"/>
+    </row>
+    <row r="202" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A202" s="47"/>
+    </row>
+    <row r="203" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A203" s="47"/>
+    </row>
+    <row r="204" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A204" s="47"/>
+    </row>
+    <row r="205" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A205" s="47"/>
+    </row>
+    <row r="206" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A206" s="47"/>
+    </row>
+    <row r="207" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A207" s="47"/>
+    </row>
+    <row r="208" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A208" s="47"/>
+    </row>
+    <row r="209" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A209" s="47"/>
+    </row>
+    <row r="210" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A210" s="47"/>
+    </row>
+    <row r="211" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A211" s="47"/>
+    </row>
+    <row r="212" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A212" s="47"/>
+    </row>
+    <row r="213" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A213" s="47"/>
+    </row>
+    <row r="214" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A214" s="47"/>
+    </row>
+    <row r="215" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A215" s="47"/>
+    </row>
+    <row r="216" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A216" s="47"/>
+    </row>
+    <row r="217" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A217" s="47"/>
+    </row>
+    <row r="218" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A218" s="47"/>
+    </row>
+    <row r="219" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A219" s="47"/>
+    </row>
+    <row r="220" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A220" s="47"/>
+    </row>
+    <row r="221" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A221" s="47"/>
+    </row>
+    <row r="222" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A222" s="47"/>
+    </row>
+    <row r="223" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A223" s="47"/>
+    </row>
+    <row r="224" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A224" s="47"/>
+    </row>
+    <row r="225" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A225" s="47"/>
+    </row>
+    <row r="226" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A226" s="47"/>
+    </row>
+    <row r="227" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A227" s="47"/>
+    </row>
+    <row r="228" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A228" s="47"/>
+    </row>
+    <row r="229" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A229" s="47"/>
+    </row>
+    <row r="230" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A230" s="47"/>
+    </row>
+    <row r="231" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A231" s="47"/>
+    </row>
+    <row r="232" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A232" s="47"/>
+    </row>
+    <row r="233" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A233" s="47"/>
+    </row>
+    <row r="234" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A234" s="47"/>
+    </row>
+    <row r="235" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A235" s="47"/>
+    </row>
+    <row r="236" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A236" s="47"/>
+    </row>
+    <row r="237" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A237" s="47"/>
+    </row>
+    <row r="238" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A238" s="47"/>
+    </row>
+    <row r="239" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A239" s="47"/>
+    </row>
+    <row r="240" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A240" s="47"/>
+    </row>
+    <row r="241" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A241" s="47"/>
+    </row>
+    <row r="242" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A242" s="47"/>
+    </row>
+    <row r="243" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A243" s="47"/>
+    </row>
+    <row r="244" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A244" s="47"/>
+    </row>
+    <row r="245" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A245" s="47"/>
+    </row>
+    <row r="246" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A246" s="47"/>
+    </row>
+    <row r="247" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A247" s="47"/>
+    </row>
+    <row r="248" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A248" s="47"/>
+    </row>
+    <row r="249" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A249" s="47"/>
+    </row>
+    <row r="250" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A250" s="47"/>
+    </row>
+    <row r="251" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A251" s="47"/>
     </row>
   </sheetData>
   <customSheetViews>
+    <customSheetView guid="{F62B73B1-1F1A-486D-90D1-651B959F68DF}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A15:E50" xr:uid="{8742F9C9-2796-4666-9D18-02DE9AC2DF21}"/>
+    </customSheetView>
     <customSheetView guid="{EB2A1D5B-713C-4666-81AF-FB92ADEAC89B}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A15:E50" xr:uid="{36F8B0F6-60CD-40CA-8DE2-F03C47AC44A3}">
+      <autoFilter ref="A15:E50" xr:uid="{3864D71A-DBAC-4EC7-B6AA-694B7D272AC6}">
         <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A15:E50">
           <sortCondition ref="B15:B50"/>
         </sortState>
       </autoFilter>
     </customSheetView>
-    <customSheetView guid="{F62B73B1-1F1A-486D-90D1-651B959F68DF}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A15:E50" xr:uid="{CDD07D98-51AD-4782-86B8-2AD65FA29937}"/>
-    </customSheetView>
   </customSheetViews>
   <phoneticPr fontId="9" type="noConversion"/>
-  <dataValidations count="3">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A7" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="C2:C7" xr:uid="{00000000-0002-0000-0000-000002000000}">
-      <formula1>AND(ISNUMBER(C2),(NOT(OR(NOT(ISERROR(DATEVALUE(C2))), AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D")))))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E70" xr:uid="{00000000-0002-0000-0000-000001000000}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E66:E128" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Matériau,Ouvrier,Divers"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2000,30 +3296,30 @@
     </row>
     <row r="3" spans="1:16" ht="22.5" customHeight="1">
       <c r="A3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="22.5" customHeight="1">
       <c r="A4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="C4" s="11">
         <v>1</v>
@@ -2036,15 +3332,15 @@
         <v>1700</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="22.5" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="11">
         <v>1</v>
@@ -2057,15 +3353,15 @@
         <v>600</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="22.5" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" s="11">
         <v>1</v>
@@ -2078,7 +3374,7 @@
         <v>1000</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="22.5" customHeight="1">
@@ -2086,7 +3382,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" s="11">
         <v>1</v>
@@ -2100,15 +3396,15 @@
         <v>499.2</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="22.5" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="11">
         <v>1</v>
@@ -2121,15 +3417,15 @@
         <v>700</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="22.5" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" s="11">
         <v>1</v>
@@ -2142,15 +3438,15 @@
         <v>500</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="22.5" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="11">
         <v>50</v>
@@ -2163,15 +3459,15 @@
         <v>40</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="22.5" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="11">
         <v>100</v>
@@ -2184,15 +3480,15 @@
         <v>80</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="22.5" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="11">
         <v>5</v>
@@ -2205,15 +3501,15 @@
         <v>75</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="22.5" customHeight="1">
       <c r="A13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="C13" s="11">
         <v>1</v>
@@ -2226,7 +3522,7 @@
         <v>60</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="22.5" customHeight="1">
@@ -2234,7 +3530,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C14" s="14">
         <v>1</v>
@@ -2247,15 +3543,15 @@
         <v>70</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="22.5" customHeight="1">
       <c r="A15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>35</v>
       </c>
       <c r="C15" s="14">
         <f>6*8*0.4*0.4</f>
@@ -2269,15 +3565,15 @@
         <v>335.6160000000001</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="22.5" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C16" s="11">
         <v>1</v>
@@ -2290,15 +3586,15 @@
         <v>981</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="22.5" customHeight="1">
       <c r="A17" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="C17" s="11">
         <v>22</v>
@@ -2311,15 +3607,15 @@
         <v>418</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="22.5" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18" s="11">
         <v>1</v>
@@ -2332,15 +3628,15 @@
         <v>107</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="22.5" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C19" s="14">
         <v>6</v>
@@ -2353,15 +3649,15 @@
         <v>96</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="22.5" customHeight="1">
       <c r="A20" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="14">
         <v>1</v>
@@ -2374,15 +3670,15 @@
         <v>22</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="22.5" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="14">
         <v>2</v>
@@ -2395,15 +3691,15 @@
         <v>24</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="22.5" customHeight="1">
       <c r="A22" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="C22" s="14">
         <v>2</v>
@@ -2416,15 +3712,15 @@
         <v>16</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="22.5" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="11">
         <v>2</v>
@@ -2437,12 +3733,12 @@
         <v>24</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="22.5" customHeight="1">
       <c r="A24" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B24" s="16"/>
       <c r="C24" s="17"/>
@@ -2458,7 +3754,7 @@
     </row>
     <row r="25" spans="1:6" ht="12.75">
       <c r="A25" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" s="6"/>
       <c r="E25" s="20">
@@ -2467,7 +3763,7 @@
     </row>
     <row r="26" spans="1:6" ht="12.75">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C26" s="6"/>
       <c r="E26" s="20">
@@ -5422,42 +6718,42 @@
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
-      <c r="K1" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
+      <c r="K1" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
     </row>
     <row r="2" spans="2:13" ht="22.5" customHeight="1">
       <c r="B2" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="D2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="H2" s="23"/>
       <c r="I2" s="23"/>
       <c r="J2" s="24"/>
       <c r="K2" s="24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L2" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="24" t="s">
         <v>50</v>
-      </c>
-      <c r="M2" s="24" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="22.5" customHeight="1">
@@ -5465,10 +6761,10 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="C3" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="27" t="s">
         <v>52</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>53</v>
       </c>
       <c r="E3" s="28">
         <v>1</v>
@@ -5499,10 +6795,10 @@
         <v>1.2</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4" s="27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E4" s="28">
         <v>1</v>
@@ -5533,10 +6829,10 @@
         <v>1.3</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5" s="28">
         <v>10</v>
@@ -5567,10 +6863,10 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="C6" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="27" t="s">
         <v>56</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>57</v>
       </c>
       <c r="E6" s="28">
         <v>4</v>
@@ -5601,10 +6897,10 @@
         <v>2.5</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D7" s="35" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E7" s="36">
         <v>1</v>
@@ -5623,7 +6919,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M7" s="32">
         <v>2500</v>
@@ -5635,7 +6931,7 @@
       <c r="D8" s="38"/>
       <c r="E8" s="38"/>
       <c r="F8" s="40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G8" s="41">
         <f>SUM(G3:G7)</f>
@@ -5646,7 +6942,7 @@
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
       <c r="L8" s="42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M8" s="43">
         <f>SUM(M3:M7)</f>
@@ -5659,7 +6955,7 @@
       <c r="D9" s="38"/>
       <c r="E9" s="38"/>
       <c r="F9" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G9" s="30">
         <f>G8*0.19</f>
@@ -5678,7 +6974,7 @@
       <c r="D10" s="38"/>
       <c r="E10" s="38"/>
       <c r="F10" s="40" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G10" s="30">
         <f>0.6</f>
@@ -5697,7 +6993,7 @@
       <c r="D11" s="38"/>
       <c r="E11" s="38"/>
       <c r="F11" s="40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G11" s="41">
         <f>+SUM(G8:G10)</f>

</xml_diff>